<commit_message>
update to light imports
</commit_message>
<xml_diff>
--- a/data/Study_dates_MeLiDos_UCR.xlsx
+++ b/data/Study_dates_MeLiDos_UCR.xlsx
@@ -1,16 +1,16 @@
 
 <file path=xl/workbook.xml><?xml version="1.0" encoding="utf-8"?>
 <workbook xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x15="http://schemas.microsoft.com/office/spreadsheetml/2010/11/main" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr6="http://schemas.microsoft.com/office/spreadsheetml/2016/revision6" xmlns:xr10="http://schemas.microsoft.com/office/spreadsheetml/2016/revision10" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" mc:Ignorable="x15 xr xr6 xr10 xr2">
-  <fileVersion appName="xl" lastEdited="7" lowestEdited="7" rupBuild="10110"/>
+  <fileVersion appName="xl" lastEdited="7" lowestEdited="7" rupBuild="10201"/>
   <workbookPr/>
   <mc:AlternateContent xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006">
     <mc:Choice Requires="x15">
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="/Users/zauner/Documents/Arbeit/12-TUM/MeLiDos/WP2.2.5_Data_Analysis/Sancho-SalasEtAl_Dataset_2025/data/"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{D60EED61-0DD3-D54B-BB4A-4830E38DF272}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{DBC072DC-783B-AB4A-A836-8CAE90C444C3}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
-    <workbookView xWindow="1300" yWindow="620" windowWidth="38200" windowHeight="22880" xr2:uid="{5E03C250-4C67-44F6-BA87-C660DAF94A8E}"/>
+    <workbookView xWindow="61520" yWindow="2300" windowWidth="38200" windowHeight="22880" xr2:uid="{5E03C250-4C67-44F6-BA87-C660DAF94A8E}"/>
   </bookViews>
   <sheets>
     <sheet name="Hoja1" sheetId="1" r:id="rId1"/>
@@ -2773,7 +2773,7 @@
         <v>45894.614583333336</v>
       </c>
       <c r="G104" s="9">
-        <v>45659.454861111109</v>
+        <v>45901.454861111109</v>
       </c>
       <c r="H104" t="s">
         <v>84</v>
@@ -2799,7 +2799,7 @@
         <v>45894.614583333336</v>
       </c>
       <c r="G105" s="9">
-        <v>45659.454861111109</v>
+        <v>45901.454861111109</v>
       </c>
       <c r="H105" t="s">
         <v>84</v>
@@ -3204,20 +3204,20 @@
 </file>
 
 <file path=customXml/item1.xml><?xml version="1.0" encoding="utf-8"?>
+<p:properties xmlns:p="http://schemas.microsoft.com/office/2006/metadata/properties" xmlns:xsi="http://www.w3.org/2001/XMLSchema-instance" xmlns:pc="http://schemas.microsoft.com/office/infopath/2007/PartnerControls">
+  <documentManagement>
+    <_activity xmlns="d5615116-53a2-4a32-b483-17fd8f718363" xsi:nil="true"/>
+  </documentManagement>
+</p:properties>
+</file>
+
+<file path=customXml/item2.xml><?xml version="1.0" encoding="utf-8"?>
 <?mso-contentType ?>
 <FormTemplates xmlns="http://schemas.microsoft.com/sharepoint/v3/contenttype/forms">
   <Display>DocumentLibraryForm</Display>
   <Edit>DocumentLibraryForm</Edit>
   <New>DocumentLibraryForm</New>
 </FormTemplates>
-</file>
-
-<file path=customXml/item2.xml><?xml version="1.0" encoding="utf-8"?>
-<p:properties xmlns:p="http://schemas.microsoft.com/office/2006/metadata/properties" xmlns:xsi="http://www.w3.org/2001/XMLSchema-instance" xmlns:pc="http://schemas.microsoft.com/office/infopath/2007/PartnerControls">
-  <documentManagement>
-    <_activity xmlns="d5615116-53a2-4a32-b483-17fd8f718363" xsi:nil="true"/>
-  </documentManagement>
-</p:properties>
 </file>
 
 <file path=customXml/item3.xml><?xml version="1.0" encoding="utf-8"?>
@@ -3460,19 +3460,19 @@
 </file>
 
 <file path=customXml/itemProps1.xml><?xml version="1.0" encoding="utf-8"?>
-<ds:datastoreItem xmlns:ds="http://schemas.openxmlformats.org/officeDocument/2006/customXml" ds:itemID="{A9546CEE-830D-4569-82E9-3186B101F743}">
+<ds:datastoreItem xmlns:ds="http://schemas.openxmlformats.org/officeDocument/2006/customXml" ds:itemID="{A1976243-C543-44E5-81C6-44C0AB7DFC98}">
   <ds:schemaRefs>
-    <ds:schemaRef ds:uri="http://schemas.microsoft.com/sharepoint/v3/contenttype/forms"/>
+    <ds:schemaRef ds:uri="http://schemas.microsoft.com/office/2006/metadata/properties"/>
+    <ds:schemaRef ds:uri="http://schemas.microsoft.com/office/infopath/2007/PartnerControls"/>
+    <ds:schemaRef ds:uri="d5615116-53a2-4a32-b483-17fd8f718363"/>
   </ds:schemaRefs>
 </ds:datastoreItem>
 </file>
 
 <file path=customXml/itemProps2.xml><?xml version="1.0" encoding="utf-8"?>
-<ds:datastoreItem xmlns:ds="http://schemas.openxmlformats.org/officeDocument/2006/customXml" ds:itemID="{A1976243-C543-44E5-81C6-44C0AB7DFC98}">
+<ds:datastoreItem xmlns:ds="http://schemas.openxmlformats.org/officeDocument/2006/customXml" ds:itemID="{A9546CEE-830D-4569-82E9-3186B101F743}">
   <ds:schemaRefs>
-    <ds:schemaRef ds:uri="http://schemas.microsoft.com/office/2006/metadata/properties"/>
-    <ds:schemaRef ds:uri="http://schemas.microsoft.com/office/infopath/2007/PartnerControls"/>
-    <ds:schemaRef ds:uri="d5615116-53a2-4a32-b483-17fd8f718363"/>
+    <ds:schemaRef ds:uri="http://schemas.microsoft.com/sharepoint/v3/contenttype/forms"/>
   </ds:schemaRefs>
 </ds:datastoreItem>
 </file>

</xml_diff>